<commit_message>
test!: formalize exchange invariants and harden residual settlement model
- add invariant test suite covering forward exchanges, loop recapture, residual attribution, and mixed-origin lots
- add expense settlement tests for residual-derived value and multi-hop unwind paths
- expand test fixture framework with BTC support and reusable exchange accounts
- formalize recursive recapture behavior through executable invariants
- verify proportional origin-basis inheritance for residual gains and losses
- verify residual settlement against inherited origin assets
- verify deterministic FIFO behavior across mixed-origin positions
- prevent uncommitted lots from affecting balances, summaries, or verification
- add committed-state tracking to UTXI and UTXO primitives
- improve account engines to ignore uncommitted ledger state
- refine REPL examples and transaction exploration workbook
- remove obsolete debugging utilities
</commit_message>
<xml_diff>
--- a/examples/transaction-exploration.xlsx
+++ b/examples/transaction-exploration.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local Storage\Repositories\Finance\Accounting-Software\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B404AF9-0F4A-4057-9803-36AA58FFC3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C25C0214-F1B1-49CA-8B5B-31E22C36784D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51495" yWindow="2805" windowWidth="19410" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51495" yWindow="3420" windowWidth="21285" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="expense-clawback" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="27">
   <si>
     <t>Cash</t>
   </si>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>USD -&gt; MXN</t>
+  </si>
+  <si>
+    <t>Hotel Expense</t>
   </si>
 </sst>
 </file>
@@ -686,6 +689,12 @@
       <c r="G5">
         <v>500</v>
       </c>
+      <c r="J5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5">
+        <v>2500</v>
+      </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
@@ -702,10 +711,41 @@
         <f>G5</f>
         <v>500</v>
       </c>
-      <c r="J6" s="1"/>
+      <c r="J6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>500</v>
+      </c>
+      <c r="F8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>250</v>
+      </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B9" s="1"/>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9">
+        <v>500</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9">
+        <f>G8</f>
+        <v>250</v>
+      </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
@@ -1685,6 +1725,10 @@
       <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="D16">
+        <f>C14*(G16/H17)</f>
+        <v>2166.6666666666665</v>
+      </c>
       <c r="F16" s="2" t="s">
         <v>14</v>
       </c>
@@ -1695,6 +1739,10 @@
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>9</v>
+      </c>
+      <c r="D17">
+        <f>C14-SUM(D15:D16)</f>
+        <v>333.33333333333394</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>0</v>

</xml_diff>